<commit_message>
Coalesce RData IDs by source so sede keeps the reviewed code and drops the SUR unit id.
RECOMENDACION_MEDIDAS_ADMIN now comes from the short measure names, and the 2026 long name no longer fills that column.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/esquema_conversion_variables_informes.xlsx
+++ b/docs/esquema_conversion_variables_informes.xlsx
@@ -1734,7 +1734,7 @@
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>IDADMIN, luego IDAMIN, luego ID_ADMIN, luego IDADMINISTRADO</t>
+          <t>IDADMINISTRADO_REV, luego IDADMIN, luego IDAMIN, luego ID_ADMIN, luego IDADMINISTRADO</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
@@ -1749,7 +1749,7 @@
       </c>
       <c r="E39" s="5" t="inlineStr">
         <is>
-          <t>Gana el primer código que ya viene lleno. En sede vigente suele ganar ID_ADMIN.</t>
+          <t>Gana el primer código que ya viene lleno. En OD solo se usa IDADMIN.</t>
         </is>
       </c>
     </row>
@@ -1788,12 +1788,12 @@
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>ID_UF, y si viene vacío IDUF_SIG</t>
+          <t>ID_UF_UNIDAD_REV, luego IDUF_SIG. El SUR de la columna ID_UF no se publica</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>IDUF_SIG</t>
+          <t>IDUF_REV, luego IDUF_SIG</t>
         </is>
       </c>
       <c r="D41" s="9" t="inlineStr">
@@ -1803,7 +1803,7 @@
       </c>
       <c r="E41" s="5" t="inlineStr">
         <is>
-          <t>En sede ID_UF es el código SUR. En OD no existe ID_UF y se usa IDUF_SIG.</t>
+          <t>En sede 2026, si no hay revisión, ID_UF queda igual a IDUF_SIG (código UF). El SUR del archivo no llega a la tabla.</t>
         </is>
       </c>
     </row>
@@ -1977,12 +1977,12 @@
       </c>
       <c r="B48" s="5" t="inlineStr">
         <is>
-          <t>RECOMENDACION DE MEDIDAS ADMINISTRATIVAS</t>
+          <t>RECOM_MA, luego RECOMENDACIÓN MEDIDAS, luego RECOM_MEDIDAS, luego RECOM_MEDIDA</t>
         </is>
       </c>
       <c r="C48" s="5" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>RECOM_MA, luego RECOMENDACIÓN MEDIDAS, luego RECOM_MEDIDAS, luego RECOM_MEDIDA</t>
         </is>
       </c>
       <c r="D48" s="9" t="inlineStr">
@@ -1992,7 +1992,7 @@
       </c>
       <c r="E48" s="5" t="inlineStr">
         <is>
-          <t>Solo sede. El espacio del nombre pasa a guion bajo.</t>
+          <t>Mismo orden en sede y OD. RECOM_MA también llena RECOM_ACCION. El nombre largo RECOMENDACION DE MEDIDAS ADMINISTRATIVAS de sede 2026 no entra; en ese corte la columna puede quedar vacía.</t>
         </is>
       </c>
     </row>
@@ -2073,7 +2073,7 @@
       </c>
       <c r="E51" s="5" t="inlineStr">
         <is>
-          <t>Se guarda tal como viene. En sede es el código UF y es distinto del SUR que queda en ID_UF. En OD coincide con ID_UF.</t>
+          <t>Se guarda tal como viene. También alimenta ID_UF. En sede el archivo trae además un SUR en la columna ID_UF, que no se publica.</t>
         </is>
       </c>
     </row>
@@ -2954,7 +2954,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E88"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3343,27 +3343,27 @@
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="15" t="inlineStr">
         <is>
           <t>SEDE</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
-        <is>
-          <t>IDADMINISTRADO_REV</t>
-        </is>
-      </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="B15" s="15" t="inlineStr">
+        <is>
+          <t>ID_SUR_UNIDAD_REV</t>
+        </is>
+      </c>
+      <c r="C15" s="15" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E15" s="5" t="inlineStr">
+      <c r="D15" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E15" s="15" t="inlineStr">
         <is>
           <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
         </is>
@@ -3377,7 +3377,7 @@
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>ID_SUR_UNIDAD_REV</t>
+          <t>TXADMINISTRADO_ADM_REV</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
@@ -3404,7 +3404,7 @@
       </c>
       <c r="B17" s="5" t="inlineStr">
         <is>
-          <t>ID_UF_UNIDAD_REV</t>
+          <t>TXUNIDAD_REV</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
@@ -3431,7 +3431,7 @@
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>TXADMINISTRADO_ADM_REV</t>
+          <t>ID</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
@@ -3446,7 +3446,7 @@
       </c>
       <c r="E18" s="15" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="B19" s="5" t="inlineStr">
         <is>
-          <t>TXUNIDAD_REV</t>
+          <t>IDACTIVIDAD</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
@@ -3473,7 +3473,7 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
         </is>
       </c>
     </row>
@@ -3485,7 +3485,7 @@
       </c>
       <c r="B20" s="15" t="inlineStr">
         <is>
-          <t>ID</t>
+          <t>IDUNIDAD</t>
         </is>
       </c>
       <c r="C20" s="15" t="inlineStr">
@@ -3512,7 +3512,7 @@
       </c>
       <c r="B21" s="5" t="inlineStr">
         <is>
-          <t>IDACTIVIDAD</t>
+          <t>RUC</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
@@ -3539,7 +3539,7 @@
       </c>
       <c r="B22" s="15" t="inlineStr">
         <is>
-          <t>IDUNIDAD</t>
+          <t>TXNUMDOC_ADM</t>
         </is>
       </c>
       <c r="C22" s="15" t="inlineStr">
@@ -3566,7 +3566,7 @@
       </c>
       <c r="B23" s="5" t="inlineStr">
         <is>
-          <t>RUC</t>
+          <t>RD_ACTA_MEDIDA</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
@@ -3581,844 +3581,844 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
+          <t>En 2019 el acta se llamaba RD_ACTA_MEDIDA. Desde el esquema vigente el mismo dato entra como RES_ACTA_MEDIDA. No se carga el nombre viejo para no duplicar la columna.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="48" customHeight="1">
-      <c r="A24" s="15" t="inlineStr">
+      <c r="A24" s="5" t="inlineStr">
         <is>
           <t>SEDE</t>
         </is>
       </c>
-      <c r="B24" s="15" t="inlineStr">
-        <is>
-          <t>TXNUMDOC_ADM</t>
-        </is>
-      </c>
-      <c r="C24" s="15" t="inlineStr">
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>VALIDADO_META</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D24" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E24" s="15" t="inlineStr">
-        <is>
-          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>Marca de validación de meta del esquema anterior. No viene en sede ni en OD de 2025/2026.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="48" customHeight="1">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="15" t="inlineStr">
         <is>
           <t>SEDE</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
-        <is>
-          <t>RD_ACTA_MEDIDA</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="B25" s="15" t="inlineStr">
+        <is>
+          <t>TXACTIVIDAD_UND</t>
+        </is>
+      </c>
+      <c r="C25" s="15" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t>En 2019 el acta se llamaba RD_ACTA_MEDIDA. Desde el esquema vigente el mismo dato entra como RES_ACTA_MEDIDA. No se carga el nombre viejo para no duplicar la columna.</t>
+      <c r="D25" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E25" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="48" customHeight="1">
-      <c r="A26" s="15" t="inlineStr">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>SEDE</t>
         </is>
       </c>
-      <c r="B26" s="15" t="inlineStr">
-        <is>
-          <t>RECOM_MEDIDA</t>
-        </is>
-      </c>
-      <c r="C26" s="15" t="inlineStr">
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>TXACTIVIDADES_VINCULADAS</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D26" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E26" s="15" t="inlineStr">
-        <is>
-          <t>En 2019 la recomendación se llamaba RECOM_MEDIDA. El nombre vigente entra como RECOMENDACION_MEDIDAS_ADMIN. El nombre corto de 2019 queda fuera.</t>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="48" customHeight="1">
-      <c r="A27" s="5" t="inlineStr">
+      <c r="A27" s="15" t="inlineStr">
         <is>
           <t>SEDE</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="15" t="inlineStr">
+        <is>
+          <t>TXCOFEMA</t>
+        </is>
+      </c>
+      <c r="C27" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D27" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E27" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="48" customHeight="1">
+      <c r="A28" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>TXDENUNCIA</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="48" customHeight="1">
+      <c r="A29" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B29" s="15" t="inlineStr">
+        <is>
+          <t>TXESTADO</t>
+        </is>
+      </c>
+      <c r="C29" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D29" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E29" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="48" customHeight="1">
+      <c r="A30" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>TXESTADO_UF</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="48" customHeight="1">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>TXETAPA_UF</t>
+        </is>
+      </c>
+      <c r="C31" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D31" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E31" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="48" customHeight="1">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>TXFUENTE</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="48" customHeight="1">
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B33" s="15" t="inlineStr">
+        <is>
+          <t>TXMES</t>
+        </is>
+      </c>
+      <c r="C33" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D33" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E33" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="48" customHeight="1">
+      <c r="A34" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>TXMOTIVOANULA</t>
+        </is>
+      </c>
+      <c r="C34" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D34" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="48" customHeight="1">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B35" s="15" t="inlineStr">
+        <is>
+          <t>TXMUESTREO</t>
+        </is>
+      </c>
+      <c r="C35" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D35" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E35" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="48" customHeight="1">
+      <c r="A36" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="inlineStr">
+        <is>
+          <t>TXNOMBRE_ANAL_LEGAL</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E36" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="48" customHeight="1">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B37" s="15" t="inlineStr">
+        <is>
+          <t>TXNOMBRE_JEFE_ACTIVIDAD</t>
+        </is>
+      </c>
+      <c r="C37" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D37" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E37" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="48" customHeight="1">
+      <c r="A38" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B38" s="5" t="inlineStr">
+        <is>
+          <t>TXNOMBRE_RESP_COMISION</t>
+        </is>
+      </c>
+      <c r="C38" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D38" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E38" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="48" customHeight="1">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B39" s="15" t="inlineStr">
+        <is>
+          <t>TXNOMBRE_RESP_MONITOREO</t>
+        </is>
+      </c>
+      <c r="C39" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D39" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E39" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="48" customHeight="1">
+      <c r="A40" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B40" s="5" t="inlineStr">
+        <is>
+          <t>TXNVL_CMPLJ</t>
+        </is>
+      </c>
+      <c r="C40" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D40" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E40" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="48" customHeight="1">
+      <c r="A41" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B41" s="15" t="inlineStr">
+        <is>
+          <t>TXOBJETIVO</t>
+        </is>
+      </c>
+      <c r="C41" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D41" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E41" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="48" customHeight="1">
+      <c r="A42" s="5" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B42" s="5" t="inlineStr">
+        <is>
+          <t>TXOTRAFUENTE</t>
+        </is>
+      </c>
+      <c r="C42" s="5" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D42" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E42" s="5" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="48" customHeight="1">
+      <c r="A43" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B43" s="15" t="inlineStr">
+        <is>
+          <t>TXUBIGEO_UND</t>
+        </is>
+      </c>
+      <c r="C43" s="15" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="D43" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E43" s="15" t="inlineStr">
+        <is>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="48" customHeight="1">
+      <c r="A44" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B44" s="5" t="inlineStr">
+        <is>
+          <t>N°</t>
+        </is>
+      </c>
+      <c r="C44" s="5" t="inlineStr">
+        <is>
+          <t>2019–2023</t>
+        </is>
+      </c>
+      <c r="D44" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E44" s="5" t="inlineStr">
+        <is>
+          <t>Es el número de fila del archivo exportado, no un dato del informe. Cambia si se vuelve a descargar el RData, así que no identifica un hecho.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45" ht="48" customHeight="1">
+      <c r="A45" s="15" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B45" s="15" t="inlineStr">
+        <is>
+          <t>COMPETENCIA</t>
+        </is>
+      </c>
+      <c r="C45" s="15" t="inlineStr">
+        <is>
+          <t>2019–2023</t>
+        </is>
+      </c>
+      <c r="D45" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E45" s="15" t="inlineStr">
+        <is>
+          <t>Hasta 2023 OD traía COMPETENCIA. Desde la plantilla vigente el campo se llama COMPET y ese sí entra a la tabla. COMPETENCIA, el nombre largo, no se carga aparte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46" ht="48" customHeight="1">
+      <c r="A46" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>ESPECIALISTA</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>2019–2021</t>
+        </is>
+      </c>
+      <c r="D46" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E46" s="5" t="inlineStr">
+        <is>
+          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47" ht="48" customHeight="1">
+      <c r="A47" s="15" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B47" s="15" t="inlineStr">
+        <is>
+          <t>JEFE</t>
+        </is>
+      </c>
+      <c r="C47" s="15" t="inlineStr">
+        <is>
+          <t>2019–2022</t>
+        </is>
+      </c>
+      <c r="D47" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E47" s="15" t="inlineStr">
+        <is>
+          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="48" ht="48" customHeight="1">
+      <c r="A48" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>FECHA_ELAB</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>2019–2021</t>
+        </is>
+      </c>
+      <c r="D48" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E48" s="5" t="inlineStr">
+        <is>
+          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="49" ht="48" customHeight="1">
+      <c r="A49" s="15" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B49" s="15" t="inlineStr">
+        <is>
+          <t>ULTIMO_DOC_ELAB</t>
+        </is>
+      </c>
+      <c r="C49" s="15" t="inlineStr">
+        <is>
+          <t>2019–2021</t>
+        </is>
+      </c>
+      <c r="D49" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E49" s="15" t="inlineStr">
+        <is>
+          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
+        </is>
+      </c>
+    </row>
+    <row r="50" ht="48" customHeight="1">
+      <c r="A50" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B50" s="5" t="inlineStr">
+        <is>
+          <t>CUENTA</t>
+        </is>
+      </c>
+      <c r="C50" s="5" t="inlineStr">
+        <is>
+          <t>2020–2021</t>
+        </is>
+      </c>
+      <c r="D50" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E50" s="5" t="inlineStr">
+        <is>
+          <t>Cuenta de usuario del sistema, no un dato del informe. Igual que USUARIO: queda para una auditoría de corrida, no para el consolidado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="51" ht="48" customHeight="1">
+      <c r="A51" s="15" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B51" s="15" t="inlineStr">
+        <is>
+          <t>MES_META_DERIV</t>
+        </is>
+      </c>
+      <c r="C51" s="15" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
+      <c r="D51" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E51" s="15" t="inlineStr">
+        <is>
+          <t>Solo aparece en OD 2021. La fecha de derivación vigente entra como FECHA_DERIV. Este nombre viejo no está en 2025/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52" ht="48" customHeight="1">
+      <c r="A52" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr">
         <is>
           <t>VALIDADO_META</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C52" s="5" t="inlineStr">
+        <is>
+          <t>2020 y 2022</t>
+        </is>
+      </c>
+      <c r="D52" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E52" s="5" t="inlineStr">
+        <is>
+          <t>Marca de validación de meta del esquema anterior. No viene en sede ni en OD de 2025/2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="53" ht="48" customHeight="1">
+      <c r="A53" s="15" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B53" s="15" t="inlineStr">
+        <is>
+          <t>ADMIN_REV</t>
+        </is>
+      </c>
+      <c r="C53" s="15" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E27" s="5" t="inlineStr">
-        <is>
-          <t>Marca de validación de meta del esquema anterior. No viene en sede ni en OD de 2025/2026.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="48" customHeight="1">
-      <c r="A28" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B28" s="15" t="inlineStr">
-        <is>
-          <t>TXACTIVIDAD_UND</t>
-        </is>
-      </c>
-      <c r="C28" s="15" t="inlineStr">
+      <c r="D53" s="15" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E53" s="15" t="inlineStr">
+        <is>
+          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" ht="48" customHeight="1">
+      <c r="A54" s="5" t="inlineStr">
+        <is>
+          <t>OD</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr">
+        <is>
+          <t>IDAMIN_REV</t>
+        </is>
+      </c>
+      <c r="C54" s="5" t="inlineStr">
         <is>
           <t>2019</t>
         </is>
       </c>
-      <c r="D28" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E28" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="48" customHeight="1">
-      <c r="A29" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B29" s="5" t="inlineStr">
-        <is>
-          <t>TXACTIVIDADES_VINCULADAS</t>
-        </is>
-      </c>
-      <c r="C29" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D29" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E29" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="48" customHeight="1">
-      <c r="A30" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B30" s="15" t="inlineStr">
-        <is>
-          <t>TXCOFEMA</t>
-        </is>
-      </c>
-      <c r="C30" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D30" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E30" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="48" customHeight="1">
-      <c r="A31" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B31" s="5" t="inlineStr">
-        <is>
-          <t>TXDENUNCIA</t>
-        </is>
-      </c>
-      <c r="C31" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D31" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E31" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="32" ht="48" customHeight="1">
-      <c r="A32" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B32" s="15" t="inlineStr">
-        <is>
-          <t>TXESTADO</t>
-        </is>
-      </c>
-      <c r="C32" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D32" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E32" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="33" ht="48" customHeight="1">
-      <c r="A33" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B33" s="5" t="inlineStr">
-        <is>
-          <t>TXESTADO_UF</t>
-        </is>
-      </c>
-      <c r="C33" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D33" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E33" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="48" customHeight="1">
-      <c r="A34" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B34" s="15" t="inlineStr">
-        <is>
-          <t>TXETAPA_UF</t>
-        </is>
-      </c>
-      <c r="C34" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D34" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E34" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="48" customHeight="1">
-      <c r="A35" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B35" s="5" t="inlineStr">
-        <is>
-          <t>TXFUENTE</t>
-        </is>
-      </c>
-      <c r="C35" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D35" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E35" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="36" ht="48" customHeight="1">
-      <c r="A36" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B36" s="15" t="inlineStr">
-        <is>
-          <t>TXMES</t>
-        </is>
-      </c>
-      <c r="C36" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D36" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E36" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="48" customHeight="1">
-      <c r="A37" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B37" s="5" t="inlineStr">
-        <is>
-          <t>TXMOTIVOANULA</t>
-        </is>
-      </c>
-      <c r="C37" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D37" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E37" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="38" ht="48" customHeight="1">
-      <c r="A38" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B38" s="15" t="inlineStr">
-        <is>
-          <t>TXMUESTREO</t>
-        </is>
-      </c>
-      <c r="C38" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D38" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E38" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="39" ht="48" customHeight="1">
-      <c r="A39" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B39" s="5" t="inlineStr">
-        <is>
-          <t>TXNOMBRE_ANAL_LEGAL</t>
-        </is>
-      </c>
-      <c r="C39" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D39" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E39" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="40" ht="48" customHeight="1">
-      <c r="A40" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B40" s="15" t="inlineStr">
-        <is>
-          <t>TXNOMBRE_JEFE_ACTIVIDAD</t>
-        </is>
-      </c>
-      <c r="C40" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D40" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E40" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41" ht="48" customHeight="1">
-      <c r="A41" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B41" s="5" t="inlineStr">
-        <is>
-          <t>TXNOMBRE_RESP_COMISION</t>
-        </is>
-      </c>
-      <c r="C41" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D41" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E41" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="42" ht="48" customHeight="1">
-      <c r="A42" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B42" s="15" t="inlineStr">
-        <is>
-          <t>TXNOMBRE_RESP_MONITOREO</t>
-        </is>
-      </c>
-      <c r="C42" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D42" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E42" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="43" ht="48" customHeight="1">
-      <c r="A43" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B43" s="5" t="inlineStr">
-        <is>
-          <t>TXNVL_CMPLJ</t>
-        </is>
-      </c>
-      <c r="C43" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D43" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E43" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="44" ht="48" customHeight="1">
-      <c r="A44" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B44" s="15" t="inlineStr">
-        <is>
-          <t>TXOBJETIVO</t>
-        </is>
-      </c>
-      <c r="C44" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D44" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E44" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="45" ht="48" customHeight="1">
-      <c r="A45" s="5" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B45" s="5" t="inlineStr">
-        <is>
-          <t>TXOTRAFUENTE</t>
-        </is>
-      </c>
-      <c r="C45" s="5" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D45" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E45" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="46" ht="48" customHeight="1">
-      <c r="A46" s="15" t="inlineStr">
-        <is>
-          <t>SEDE</t>
-        </is>
-      </c>
-      <c r="B46" s="15" t="inlineStr">
-        <is>
-          <t>TXUBIGEO_UND</t>
-        </is>
-      </c>
-      <c r="C46" s="15" t="inlineStr">
-        <is>
-          <t>2019</t>
-        </is>
-      </c>
-      <c r="D46" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E46" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="47" ht="48" customHeight="1">
-      <c r="A47" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B47" s="5" t="inlineStr">
-        <is>
-          <t>N°</t>
-        </is>
-      </c>
-      <c r="C47" s="5" t="inlineStr">
-        <is>
-          <t>2019–2023</t>
-        </is>
-      </c>
-      <c r="D47" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E47" s="5" t="inlineStr">
-        <is>
-          <t>Es el número de fila del archivo exportado, no un dato del informe. Cambia si se vuelve a descargar el RData, así que no identifica un hecho.</t>
-        </is>
-      </c>
-    </row>
-    <row r="48" ht="48" customHeight="1">
-      <c r="A48" s="15" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B48" s="15" t="inlineStr">
-        <is>
-          <t>COMPETENCIA</t>
-        </is>
-      </c>
-      <c r="C48" s="15" t="inlineStr">
-        <is>
-          <t>2019–2023</t>
-        </is>
-      </c>
-      <c r="D48" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E48" s="15" t="inlineStr">
-        <is>
-          <t>Hasta 2023 OD traía COMPETENCIA. Desde la plantilla vigente el campo se llama COMPET y ese sí entra a la tabla. COMPETENCIA, el nombre largo, no se carga aparte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="49" ht="48" customHeight="1">
-      <c r="A49" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr">
-        <is>
-          <t>ESPECIALISTA</t>
-        </is>
-      </c>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>2019–2021</t>
-        </is>
-      </c>
-      <c r="D49" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E49" s="5" t="inlineStr">
-        <is>
-          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
-        </is>
-      </c>
-    </row>
-    <row r="50" ht="48" customHeight="1">
-      <c r="A50" s="15" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B50" s="15" t="inlineStr">
-        <is>
-          <t>JEFE</t>
-        </is>
-      </c>
-      <c r="C50" s="15" t="inlineStr">
-        <is>
-          <t>2019–2022</t>
-        </is>
-      </c>
-      <c r="D50" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E50" s="15" t="inlineStr">
-        <is>
-          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
-        </is>
-      </c>
-    </row>
-    <row r="51" ht="48" customHeight="1">
-      <c r="A51" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr">
-        <is>
-          <t>FECHA_ELAB</t>
-        </is>
-      </c>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>2019–2021</t>
-        </is>
-      </c>
-      <c r="D51" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E51" s="5" t="inlineStr">
-        <is>
-          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
-        </is>
-      </c>
-    </row>
-    <row r="52" ht="48" customHeight="1">
-      <c r="A52" s="15" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B52" s="15" t="inlineStr">
-        <is>
-          <t>ULTIMO_DOC_ELAB</t>
-        </is>
-      </c>
-      <c r="C52" s="15" t="inlineStr">
-        <is>
-          <t>2019–2021</t>
-        </is>
-      </c>
-      <c r="D52" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E52" s="15" t="inlineStr">
-        <is>
-          <t>Campo de los OD antiguos (especialista, jefe o documento de elaboración). Los archivos OD de 2025 y 2026 ya no lo traen, así que en el corte que se consume quedaría vacío.</t>
-        </is>
-      </c>
-    </row>
-    <row r="53" ht="48" customHeight="1">
-      <c r="A53" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B53" s="5" t="inlineStr">
-        <is>
-          <t>CUENTA</t>
-        </is>
-      </c>
-      <c r="C53" s="5" t="inlineStr">
-        <is>
-          <t>2020–2021</t>
-        </is>
-      </c>
-      <c r="D53" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E53" s="5" t="inlineStr">
-        <is>
-          <t>Cuenta de usuario del sistema, no un dato del informe. Igual que USUARIO: queda para una auditoría de corrida, no para el consolidado.</t>
-        </is>
-      </c>
-    </row>
-    <row r="54" ht="48" customHeight="1">
-      <c r="A54" s="15" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B54" s="15" t="inlineStr">
-        <is>
-          <t>MES_META_DERIV</t>
-        </is>
-      </c>
-      <c r="C54" s="15" t="inlineStr">
-        <is>
-          <t>2021</t>
-        </is>
-      </c>
-      <c r="D54" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E54" s="15" t="inlineStr">
-        <is>
-          <t>Solo aparece en OD 2021. La fecha de derivación vigente entra como FECHA_DERIV. Este nombre viejo no está en 2025/2026.</t>
+      <c r="D54" s="5" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="E54" s="5" t="inlineStr">
+        <is>
+          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
         </is>
       </c>
     </row>
@@ -4430,12 +4430,12 @@
       </c>
       <c r="B55" s="5" t="inlineStr">
         <is>
-          <t>VALIDADO_META</t>
+          <t>UF_REV</t>
         </is>
       </c>
       <c r="C55" s="5" t="inlineStr">
         <is>
-          <t>2020 y 2022</t>
+          <t>2019</t>
         </is>
       </c>
       <c r="D55" s="5" t="inlineStr">
@@ -4445,7 +4445,7 @@
       </c>
       <c r="E55" s="5" t="inlineStr">
         <is>
-          <t>Marca de validación de meta del esquema anterior. No viene en sede ni en OD de 2025/2026.</t>
+          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
         </is>
       </c>
     </row>
@@ -4457,12 +4457,12 @@
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>ADMIN_REV</t>
+          <t>FEANUL_SIIA</t>
         </is>
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D56" s="15" t="inlineStr">
@@ -4472,7 +4472,7 @@
       </c>
       <c r="E56" s="15" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
         </is>
       </c>
     </row>
@@ -4484,12 +4484,12 @@
       </c>
       <c r="B57" s="5" t="inlineStr">
         <is>
-          <t>IDAMIN_REV</t>
+          <t>FEAPROB_SIIA</t>
         </is>
       </c>
       <c r="C57" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D57" s="5" t="inlineStr">
@@ -4499,7 +4499,7 @@
       </c>
       <c r="E57" s="5" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
         </is>
       </c>
     </row>
@@ -4511,12 +4511,12 @@
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>IDUF_REV</t>
+          <t>FEREG_SIIA</t>
         </is>
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D58" s="15" t="inlineStr">
@@ -4526,7 +4526,7 @@
       </c>
       <c r="E58" s="15" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
         </is>
       </c>
     </row>
@@ -4538,12 +4538,12 @@
       </c>
       <c r="B59" s="5" t="inlineStr">
         <is>
-          <t>UF_REV</t>
+          <t>FERPT</t>
         </is>
       </c>
       <c r="C59" s="5" t="inlineStr">
         <is>
-          <t>2019</t>
+          <t>2020</t>
         </is>
       </c>
       <c r="D59" s="5" t="inlineStr">
@@ -4553,7 +4553,7 @@
       </c>
       <c r="E59" s="5" t="inlineStr">
         <is>
-          <t>Es un espejo del mismo dato con sufijo _REV (copia de revisión). El valor de negocio ya entra por la columna principal (administrado, unidad o UF). Esta copia no agrega un hecho nuevo.</t>
+          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
         </is>
       </c>
     </row>
@@ -4565,7 +4565,7 @@
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>FEANUL_SIIA</t>
+          <t>FGSUPUPD_1ERTIEMPO</t>
         </is>
       </c>
       <c r="C60" s="15" t="inlineStr">
@@ -4580,7 +4580,7 @@
       </c>
       <c r="E60" s="15" t="inlineStr">
         <is>
-          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
+          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
         </is>
       </c>
     </row>
@@ -4592,7 +4592,7 @@
       </c>
       <c r="B61" s="5" t="inlineStr">
         <is>
-          <t>FEAPROB_SIIA</t>
+          <t>FGSUPUPD_2DOTIEMPO</t>
         </is>
       </c>
       <c r="C61" s="5" t="inlineStr">
@@ -4607,7 +4607,7 @@
       </c>
       <c r="E61" s="5" t="inlineStr">
         <is>
-          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
+          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
         </is>
       </c>
     </row>
@@ -4619,7 +4619,7 @@
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>FEREG_SIIA</t>
+          <t>FGSUP_ORIENTATIVA</t>
         </is>
       </c>
       <c r="C62" s="15" t="inlineStr">
@@ -4634,7 +4634,7 @@
       </c>
       <c r="E62" s="15" t="inlineStr">
         <is>
-          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
+          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
         </is>
       </c>
     </row>
@@ -4646,7 +4646,7 @@
       </c>
       <c r="B63" s="5" t="inlineStr">
         <is>
-          <t>FERPT</t>
+          <t>IDACTIVIDAD</t>
         </is>
       </c>
       <c r="C63" s="5" t="inlineStr">
@@ -4661,7 +4661,7 @@
       </c>
       <c r="E63" s="5" t="inlineStr">
         <is>
-          <t>Fecha del sistema anterior (SIIA). Solo aparece en 2019 o 2020. En la plantilla 2025/2026 el archivo ya no trae esta columna, así que en los cortes actuales quedaría siempre vacía.</t>
+          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
         </is>
       </c>
     </row>
@@ -4673,7 +4673,7 @@
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>FGSUPUPD_1ERTIEMPO</t>
+          <t>IDUNIDAD</t>
         </is>
       </c>
       <c r="C64" s="15" t="inlineStr">
@@ -4688,7 +4688,7 @@
       </c>
       <c r="E64" s="15" t="inlineStr">
         <is>
-          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
+          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
         </is>
       </c>
     </row>
@@ -4700,7 +4700,7 @@
       </c>
       <c r="B65" s="5" t="inlineStr">
         <is>
-          <t>FGSUPUPD_2DOTIEMPO</t>
+          <t>TXNUMDOC_ADM</t>
         </is>
       </c>
       <c r="C65" s="5" t="inlineStr">
@@ -4715,7 +4715,7 @@
       </c>
       <c r="E65" s="5" t="inlineStr">
         <is>
-          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
+          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>FGSUP_ORIENTATIVA</t>
+          <t>TXACTIVIDAD_UND</t>
         </is>
       </c>
       <c r="C66" s="15" t="inlineStr">
@@ -4742,7 +4742,7 @@
       </c>
       <c r="E66" s="15" t="inlineStr">
         <is>
-          <t>Indicador del esquema SIIA. No está en los RData de 2025 ni de 2026. Cargarlo dejaría la columna vacía en todo el corte que se consume.</t>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
@@ -4754,7 +4754,7 @@
       </c>
       <c r="B67" s="5" t="inlineStr">
         <is>
-          <t>IDACTIVIDAD</t>
+          <t>TXACTIVIDADES_VINCULADAS</t>
         </is>
       </c>
       <c r="C67" s="5" t="inlineStr">
@@ -4769,7 +4769,7 @@
       </c>
       <c r="E67" s="5" t="inlineStr">
         <is>
-          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
@@ -4781,7 +4781,7 @@
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>IDUNIDAD</t>
+          <t>TXCOFEMA</t>
         </is>
       </c>
       <c r="C68" s="15" t="inlineStr">
@@ -4796,7 +4796,7 @@
       </c>
       <c r="E68" s="15" t="inlineStr">
         <is>
-          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
@@ -4808,7 +4808,7 @@
       </c>
       <c r="B69" s="5" t="inlineStr">
         <is>
-          <t>TXNUMDOC_ADM</t>
+          <t>TXDENUNCIA</t>
         </is>
       </c>
       <c r="C69" s="5" t="inlineStr">
@@ -4823,7 +4823,7 @@
       </c>
       <c r="E69" s="5" t="inlineStr">
         <is>
-          <t>Código interno del esquema SIIA (actividad, unidad, RUC u otro id viejo). No está en la plantilla vigente y no es el ID_ADMINISTRADO ni el ID_UF que sí se guardan.</t>
+          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
         </is>
       </c>
     </row>
@@ -4835,7 +4835,7 @@
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>TXACTIVIDAD_UND</t>
+          <t>TXESTADO</t>
         </is>
       </c>
       <c r="C70" s="15" t="inlineStr">
@@ -4862,7 +4862,7 @@
       </c>
       <c r="B71" s="5" t="inlineStr">
         <is>
-          <t>TXACTIVIDADES_VINCULADAS</t>
+          <t>TXESTADO_UF</t>
         </is>
       </c>
       <c r="C71" s="5" t="inlineStr">
@@ -4889,7 +4889,7 @@
       </c>
       <c r="B72" s="15" t="inlineStr">
         <is>
-          <t>TXCOFEMA</t>
+          <t>TXETAPA_UF</t>
         </is>
       </c>
       <c r="C72" s="15" t="inlineStr">
@@ -4916,7 +4916,7 @@
       </c>
       <c r="B73" s="5" t="inlineStr">
         <is>
-          <t>TXDENUNCIA</t>
+          <t>TXFUENTE</t>
         </is>
       </c>
       <c r="C73" s="5" t="inlineStr">
@@ -4943,7 +4943,7 @@
       </c>
       <c r="B74" s="15" t="inlineStr">
         <is>
-          <t>TXESTADO</t>
+          <t>TXMES</t>
         </is>
       </c>
       <c r="C74" s="15" t="inlineStr">
@@ -4970,7 +4970,7 @@
       </c>
       <c r="B75" s="5" t="inlineStr">
         <is>
-          <t>TXESTADO_UF</t>
+          <t>TXMOTIVOANULA</t>
         </is>
       </c>
       <c r="C75" s="5" t="inlineStr">
@@ -4997,7 +4997,7 @@
       </c>
       <c r="B76" s="15" t="inlineStr">
         <is>
-          <t>TXETAPA_UF</t>
+          <t>TXMUESTREO</t>
         </is>
       </c>
       <c r="C76" s="15" t="inlineStr">
@@ -5024,7 +5024,7 @@
       </c>
       <c r="B77" s="5" t="inlineStr">
         <is>
-          <t>TXFUENTE</t>
+          <t>TXNOMBRE_ANAL_LEGAL</t>
         </is>
       </c>
       <c r="C77" s="5" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="B78" s="15" t="inlineStr">
         <is>
-          <t>TXMES</t>
+          <t>TXNOMBRE_JEFE_ACTIVIDAD</t>
         </is>
       </c>
       <c r="C78" s="15" t="inlineStr">
@@ -5078,7 +5078,7 @@
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>TXMOTIVOANULA</t>
+          <t>TXNOMBRE_RESP_COMISION</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
@@ -5105,7 +5105,7 @@
       </c>
       <c r="B80" s="15" t="inlineStr">
         <is>
-          <t>TXMUESTREO</t>
+          <t>TXNOMBRE_RESP_MONITOREO</t>
         </is>
       </c>
       <c r="C80" s="15" t="inlineStr">
@@ -5132,7 +5132,7 @@
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>TXNOMBRE_ANAL_LEGAL</t>
+          <t>TXNVL_CMPLJ</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
@@ -5159,7 +5159,7 @@
       </c>
       <c r="B82" s="15" t="inlineStr">
         <is>
-          <t>TXNOMBRE_JEFE_ACTIVIDAD</t>
+          <t>TXOBJETIVO</t>
         </is>
       </c>
       <c r="C82" s="15" t="inlineStr">
@@ -5186,7 +5186,7 @@
       </c>
       <c r="B83" s="5" t="inlineStr">
         <is>
-          <t>TXNOMBRE_RESP_COMISION</t>
+          <t>TXOTRAFUENTE</t>
         </is>
       </c>
       <c r="C83" s="5" t="inlineStr">
@@ -5213,7 +5213,7 @@
       </c>
       <c r="B84" s="15" t="inlineStr">
         <is>
-          <t>TXNOMBRE_RESP_MONITOREO</t>
+          <t>TXUBIGEO_UND</t>
         </is>
       </c>
       <c r="C84" s="15" t="inlineStr">
@@ -5233,113 +5233,61 @@
       </c>
     </row>
     <row r="85" ht="48" customHeight="1">
-      <c r="A85" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B85" s="5" t="inlineStr">
-        <is>
-          <t>TXNVL_CMPLJ</t>
-        </is>
-      </c>
-      <c r="C85" s="5" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="D85" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E85" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
+      <c r="A85" s="15" t="inlineStr">
+        <is>
+          <t>SEDE</t>
+        </is>
+      </c>
+      <c r="B85" s="15" t="inlineStr">
+        <is>
+          <t>ID_UF (código SUR)</t>
+        </is>
+      </c>
+      <c r="C85" s="15" t="inlineStr">
+        <is>
+          <t>2019–2026</t>
+        </is>
+      </c>
+      <c r="D85" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="E85" s="15" t="inlineStr">
+        <is>
+          <t>La columna del archivo llamada ID_UF trae el código SUR. Ya no se publica. La columna ID_UF de la tabla sale de ID_UF_UNIDAD_REV y de IDUF_SIG.</t>
         </is>
       </c>
     </row>
     <row r="86" ht="48" customHeight="1">
       <c r="A86" s="15" t="inlineStr">
         <is>
-          <t>OD</t>
+          <t>SEDE</t>
         </is>
       </c>
       <c r="B86" s="15" t="inlineStr">
         <is>
-          <t>TXOBJETIVO</t>
+          <t>RECOMENDACION DE MEDIDAS ADMINISTRATIVAS</t>
         </is>
       </c>
       <c r="C86" s="15" t="inlineStr">
         <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="D86" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="D86" s="16" t="inlineStr">
+        <is>
+          <t>Sí</t>
         </is>
       </c>
       <c r="E86" s="15" t="inlineStr">
         <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="87" ht="48" customHeight="1">
-      <c r="A87" s="5" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B87" s="5" t="inlineStr">
-        <is>
-          <t>TXOTRAFUENTE</t>
-        </is>
-      </c>
-      <c r="C87" s="5" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="D87" s="5" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E87" s="5" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="88" ht="48" customHeight="1">
-      <c r="A88" s="15" t="inlineStr">
-        <is>
-          <t>OD</t>
-        </is>
-      </c>
-      <c r="B88" s="15" t="inlineStr">
-        <is>
-          <t>TXUBIGEO_UND</t>
-        </is>
-      </c>
-      <c r="C88" s="15" t="inlineStr">
-        <is>
-          <t>2020</t>
-        </is>
-      </c>
-      <c r="D88" s="15" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="E88" s="15" t="inlineStr">
-        <is>
-          <t>Texto del sistema anterior: estado, fuente, objetivo, ubigeo, denuncia, muestreo o nombre de responsable. El bloque completo desaparece en la plantilla 2025/2026. En los cortes actuales no hay columna que llenar.</t>
-        </is>
-      </c>
-    </row>
+          <t>Es el nombre vigente en sede 2026. Ya no alimenta RECOMENDACION_MEDIDAS_ADMIN. Esa columna se llena con RECOM_MA, RECOMENDACIÓN MEDIDAS, RECOM_MEDIDAS y RECOM_MEDIDA.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" ht="48" customHeight="1"/>
+    <row r="88" ht="48" customHeight="1"/>
   </sheetData>
   <autoFilter ref="A1:E88"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>